<commit_message>
TARSP report improvements and WVz improvement
</commit_message>
<xml_diff>
--- a/src/sastadev/data/methods/TARSP_Index_Current.xlsx
+++ b/src/sastadev/data/methods/TARSP_Index_Current.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\jodijk\myprograms\python\sastacode\mysastadev\src\sastadev\data\methods\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2398EB5A-A47C-4320-9FB4-0AEAA112EF13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8F0F7D2-8CCF-4DC7-8E76-3FC5E04EEE31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$Y$159</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$Y$166</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -1548,9 +1548,6 @@
     <t>Znx</t>
   </si>
   <si>
-    <t>//node[node[@pt="ww"  and @rel ="hd"] and node[@rel="pc" and not(%Tarsp_B%)]]</t>
-  </si>
-  <si>
     <t>//node[%complement% and parent::node[(@cat="smain" or @cat="sv1" or @cat="ssub" or @cat="inf" or @cat="ppart") ]]</t>
   </si>
   <si>
@@ -2169,6 +2166,9 @@
   </si>
   <si>
     <t>//node[(@cat="ap" or @cat="advp") and node[(@rel="mod" or @rel="me") and @cat="np" and node[@rel="det"]]]</t>
+  </si>
+  <si>
+    <t>//node[@pt="ww"  and @rel ="hd" and ../node[@rel="pc" and not(%Tarsp_B%)]]</t>
   </si>
 </sst>
 </file>
@@ -2255,23 +2255,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
@@ -2604,7 +2601,7 @@
     <col min="12" max="12" width="41.109375" style="2" customWidth="1"/>
     <col min="13" max="13" width="9" style="2" bestFit="1" customWidth="1"/>
     <col min="14" max="19" width="16.21875" style="2" customWidth="1"/>
-    <col min="20" max="20" width="16.21875" style="15" customWidth="1"/>
+    <col min="20" max="20" width="16.21875" style="12" customWidth="1"/>
     <col min="21" max="23" width="16.21875" style="2" customWidth="1"/>
     <col min="24" max="16384" width="8.88671875" style="2"/>
   </cols>
@@ -2635,10 +2632,10 @@
         <v>350</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>624</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>625</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>626</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>41</v>
@@ -2656,28 +2653,28 @@
         <v>434</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="Q1" s="1" t="s">
+        <v>536</v>
+      </c>
+      <c r="R1" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>538</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="11" t="s">
+        <v>626</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>627</v>
+      </c>
+      <c r="V1" s="1" t="s">
         <v>539</v>
       </c>
-      <c r="T1" s="14" t="s">
-        <v>627</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>628</v>
-      </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>540</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>541</v>
       </c>
       <c r="X1" s="1" t="s">
         <v>157</v>
@@ -2697,13 +2694,13 @@
         <v>191</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>69</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>351</v>
@@ -2715,7 +2712,7 @@
         <v>3</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="M2" s="2" t="s">
         <v>351</v>
@@ -2730,7 +2727,7 @@
         <v>446</v>
       </c>
       <c r="T2" s="2" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.3">
@@ -2771,7 +2768,7 @@
         <v>435</v>
       </c>
       <c r="T3" s="2" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="X3" s="2" t="s">
         <v>419</v>
@@ -2815,10 +2812,10 @@
         <v>435</v>
       </c>
       <c r="S4" s="2" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="T4" s="2" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.3">
@@ -2856,7 +2853,7 @@
         <v>435</v>
       </c>
       <c r="T5" s="2" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="X5" s="2" t="s">
         <v>183</v>
@@ -2885,7 +2882,7 @@
         <v>1</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="M6" s="2" t="s">
         <v>351</v>
@@ -2896,8 +2893,8 @@
       <c r="O6" s="2" t="s">
         <v>435</v>
       </c>
-      <c r="T6" s="15" t="s">
-        <v>672</v>
+      <c r="T6" s="12" t="s">
+        <v>671</v>
       </c>
       <c r="X6" s="2" t="s">
         <v>357</v>
@@ -2917,7 +2914,7 @@
         <v>191</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>351</v>
@@ -3007,7 +3004,7 @@
         <v>6</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="M9" s="2" t="s">
         <v>351</v>
@@ -3019,7 +3016,7 @@
         <v>435</v>
       </c>
       <c r="T9" s="2" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="X9" s="2" t="s">
         <v>367</v>
@@ -3048,7 +3045,7 @@
         <v>4</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="M10" s="3" t="s">
         <v>351</v>
@@ -3060,7 +3057,7 @@
         <v>435</v>
       </c>
       <c r="T10" s="2" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.3">
@@ -3116,7 +3113,7 @@
         <v>37</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>351</v>
@@ -3128,7 +3125,7 @@
         <v>3</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="M12" s="2" t="s">
         <v>351</v>
@@ -3140,7 +3137,7 @@
         <v>435</v>
       </c>
       <c r="T12" s="2" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.3">
@@ -3166,7 +3163,7 @@
         <v>5</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="M13" s="3" t="s">
         <v>351</v>
@@ -3178,7 +3175,7 @@
         <v>435</v>
       </c>
       <c r="T13" s="2" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.3">
@@ -3207,7 +3204,7 @@
         <v>4</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="M14" s="2" t="s">
         <v>352</v>
@@ -3243,7 +3240,7 @@
         <v>4</v>
       </c>
       <c r="L15" s="3" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="M15" s="2" t="s">
         <v>351</v>
@@ -3255,7 +3252,7 @@
         <v>435</v>
       </c>
       <c r="T15" s="2" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.3">
@@ -3362,7 +3359,7 @@
         <v>446</v>
       </c>
       <c r="T18" s="2" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.3">
@@ -3379,7 +3376,7 @@
         <v>383</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="H19" s="2" t="s">
         <v>351</v>
@@ -3391,7 +3388,7 @@
         <v>1</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="M19" s="2" t="s">
         <v>351</v>
@@ -3402,8 +3399,8 @@
       <c r="O19" s="2" t="s">
         <v>435</v>
       </c>
-      <c r="T19" s="15" t="s">
-        <v>673</v>
+      <c r="T19" s="12" t="s">
+        <v>672</v>
       </c>
     </row>
     <row r="20" spans="1:24" x14ac:dyDescent="0.3">
@@ -3438,7 +3435,7 @@
         <v>435</v>
       </c>
       <c r="T20" s="2" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
     </row>
     <row r="21" spans="1:24" x14ac:dyDescent="0.3">
@@ -3464,7 +3461,7 @@
         <v>4</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="M21" s="2" t="s">
         <v>351</v>
@@ -3476,7 +3473,7 @@
         <v>435</v>
       </c>
       <c r="T21" s="2" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
     </row>
     <row r="22" spans="1:24" x14ac:dyDescent="0.3">
@@ -3514,7 +3511,7 @@
         <v>435</v>
       </c>
       <c r="T22" s="2" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="U22" s="2" t="s">
         <v>222</v>
@@ -3537,7 +3534,7 @@
         <v>46</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="H23" s="2" t="s">
         <v>351</v>
@@ -3549,7 +3546,7 @@
         <v>5</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="M23" s="2" t="s">
         <v>351</v>
@@ -3561,7 +3558,7 @@
         <v>435</v>
       </c>
       <c r="T23" s="2" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
     </row>
     <row r="24" spans="1:24" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -3584,7 +3581,7 @@
         <v>25</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="H24" s="2" t="s">
         <v>351</v>
@@ -3596,7 +3593,7 @@
         <v>2</v>
       </c>
       <c r="L24" s="3" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="M24" s="2" t="s">
         <v>351</v>
@@ -3608,7 +3605,7 @@
         <v>435</v>
       </c>
       <c r="T24" s="2" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="U24" s="2" t="s">
         <v>221</v>
@@ -3673,7 +3670,7 @@
         <v>4</v>
       </c>
       <c r="L26" s="3" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="M26" s="3" t="s">
         <v>351</v>
@@ -3685,7 +3682,7 @@
         <v>435</v>
       </c>
       <c r="T26" s="2" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="X26" s="2" t="s">
         <v>469</v>
@@ -3714,7 +3711,7 @@
         <v>4</v>
       </c>
       <c r="L27" s="3" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="M27" s="2" t="s">
         <v>351</v>
@@ -3726,7 +3723,7 @@
         <v>435</v>
       </c>
       <c r="T27" s="2" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
     </row>
     <row r="28" spans="1:24" x14ac:dyDescent="0.3">
@@ -3752,7 +3749,7 @@
         <v>5</v>
       </c>
       <c r="L28" s="2" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="M28" s="2" t="s">
         <v>351</v>
@@ -3764,7 +3761,7 @@
         <v>435</v>
       </c>
       <c r="T28" s="2" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
     </row>
     <row r="29" spans="1:24" x14ac:dyDescent="0.3">
@@ -3790,7 +3787,7 @@
         <v>2</v>
       </c>
       <c r="L29" s="2" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="M29" s="2" t="s">
         <v>351</v>
@@ -3802,7 +3799,7 @@
         <v>435</v>
       </c>
       <c r="T29" s="2" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="X29" s="2" t="s">
         <v>365</v>
@@ -3831,7 +3828,7 @@
         <v>3</v>
       </c>
       <c r="L30" s="2" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="M30" s="2" t="s">
         <v>351</v>
@@ -3843,7 +3840,7 @@
         <v>435</v>
       </c>
       <c r="T30" s="2" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="X30" s="2" t="s">
         <v>183</v>
@@ -3884,10 +3881,10 @@
         <v>435</v>
       </c>
       <c r="S31" s="2" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="T31" s="2" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
     </row>
     <row r="32" spans="1:24" x14ac:dyDescent="0.3">
@@ -3916,7 +3913,7 @@
         <v>6</v>
       </c>
       <c r="L32" s="3" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="M32" s="3" t="s">
         <v>351</v>
@@ -3928,7 +3925,7 @@
         <v>435</v>
       </c>
       <c r="T32" s="2" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
     </row>
     <row r="33" spans="1:24" x14ac:dyDescent="0.3">
@@ -3960,7 +3957,7 @@
         <v>3</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="M33" s="2" t="s">
         <v>351</v>
@@ -3972,10 +3969,10 @@
         <v>435</v>
       </c>
       <c r="S33" s="2" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="T33" s="2" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
     </row>
     <row r="34" spans="1:24" x14ac:dyDescent="0.3">
@@ -4001,7 +3998,7 @@
         <v>6</v>
       </c>
       <c r="L34" s="2" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="M34" s="2" t="s">
         <v>351</v>
@@ -4013,7 +4010,7 @@
         <v>435</v>
       </c>
       <c r="T34" s="2" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
     </row>
     <row r="35" spans="1:24" x14ac:dyDescent="0.3">
@@ -4051,7 +4048,7 @@
         <v>435</v>
       </c>
       <c r="T35" s="2" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
     </row>
     <row r="36" spans="1:24" x14ac:dyDescent="0.3">
@@ -4077,7 +4074,7 @@
         <v>5</v>
       </c>
       <c r="L36" s="3" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="M36" s="3" t="s">
         <v>351</v>
@@ -4089,7 +4086,7 @@
         <v>435</v>
       </c>
       <c r="T36" s="2" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
     </row>
     <row r="37" spans="1:24" x14ac:dyDescent="0.3">
@@ -4115,7 +4112,7 @@
         <v>3</v>
       </c>
       <c r="L37" s="2" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="M37" s="2" t="s">
         <v>351</v>
@@ -4127,7 +4124,7 @@
         <v>435</v>
       </c>
       <c r="T37" s="2" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
     </row>
     <row r="38" spans="1:24" x14ac:dyDescent="0.3">
@@ -4147,7 +4144,7 @@
         <v>207</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="H38" s="2" t="s">
         <v>351</v>
@@ -4159,7 +4156,7 @@
         <v>361</v>
       </c>
       <c r="L38" s="3" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="M38" s="3" t="s">
         <v>351</v>
@@ -4171,7 +4168,7 @@
         <v>435</v>
       </c>
       <c r="T38" s="2" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
     </row>
     <row r="39" spans="1:24" x14ac:dyDescent="0.3">
@@ -4191,7 +4188,7 @@
         <v>208</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="H39" s="2" t="s">
         <v>351</v>
@@ -4203,7 +4200,7 @@
         <v>4</v>
       </c>
       <c r="L39" s="3" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="M39" s="3" t="s">
         <v>351</v>
@@ -4215,7 +4212,7 @@
         <v>435</v>
       </c>
       <c r="T39" s="2" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
     </row>
     <row r="40" spans="1:24" x14ac:dyDescent="0.3">
@@ -4232,7 +4229,7 @@
         <v>144</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="H40" s="2" t="s">
         <v>351</v>
@@ -4256,7 +4253,7 @@
         <v>435</v>
       </c>
       <c r="T40" s="2" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="X40" s="2" t="s">
         <v>470</v>
@@ -4297,7 +4294,7 @@
         <v>435</v>
       </c>
       <c r="T41" s="2" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
     </row>
     <row r="42" spans="1:24" x14ac:dyDescent="0.3">
@@ -4329,7 +4326,7 @@
         <v>2</v>
       </c>
       <c r="L42" s="2" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="M42" s="2" t="s">
         <v>351</v>
@@ -4341,7 +4338,7 @@
         <v>435</v>
       </c>
       <c r="T42" s="2" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="X42" s="2" t="s">
         <v>160</v>
@@ -4376,7 +4373,7 @@
         <v>3</v>
       </c>
       <c r="L43" s="3" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="M43" s="2" t="s">
         <v>351</v>
@@ -4388,7 +4385,7 @@
         <v>435</v>
       </c>
       <c r="T43" s="2" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="X43" s="2" t="s">
         <v>356</v>
@@ -4417,7 +4414,7 @@
         <v>3</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="M44" s="2" t="s">
         <v>351</v>
@@ -4429,7 +4426,7 @@
         <v>435</v>
       </c>
       <c r="T44" s="2" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
     </row>
     <row r="45" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
@@ -4467,7 +4464,7 @@
         <v>435</v>
       </c>
       <c r="T45" s="2" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
     </row>
     <row r="46" spans="1:24" x14ac:dyDescent="0.3">
@@ -4490,7 +4487,7 @@
         <v>200</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="H46" s="2" t="s">
         <v>351</v>
@@ -4514,7 +4511,7 @@
         <v>435</v>
       </c>
       <c r="T46" s="2" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
     </row>
     <row r="47" spans="1:24" ht="86.4" x14ac:dyDescent="0.3">
@@ -4552,7 +4549,7 @@
         <v>435</v>
       </c>
       <c r="T47" s="2" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="X47" s="2" t="s">
         <v>183</v>
@@ -4572,7 +4569,7 @@
         <v>352</v>
       </c>
       <c r="L48" s="3" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="M48" s="3" t="s">
         <v>352</v>
@@ -4584,7 +4581,7 @@
         <v>435</v>
       </c>
       <c r="T48" s="2"/>
-      <c r="X48" s="6" t="s">
+      <c r="X48" s="2" t="s">
         <v>178</v>
       </c>
     </row>
@@ -4659,7 +4656,7 @@
         <v>435</v>
       </c>
       <c r="T50" s="2" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
     </row>
     <row r="51" spans="1:24" x14ac:dyDescent="0.3">
@@ -4685,7 +4682,7 @@
         <v>4</v>
       </c>
       <c r="L51" s="2" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="M51" s="2" t="s">
         <v>351</v>
@@ -4697,7 +4694,7 @@
         <v>435</v>
       </c>
       <c r="T51" s="2" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
     </row>
     <row r="52" spans="1:24" x14ac:dyDescent="0.3">
@@ -4726,7 +4723,7 @@
         <v>2</v>
       </c>
       <c r="L52" s="2" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="M52" s="2" t="s">
         <v>351</v>
@@ -4738,7 +4735,7 @@
         <v>435</v>
       </c>
       <c r="T52" s="2" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
     </row>
     <row r="53" spans="1:24" x14ac:dyDescent="0.3">
@@ -4764,7 +4761,7 @@
         <v>6</v>
       </c>
       <c r="L53" s="2" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="M53" s="2" t="s">
         <v>351</v>
@@ -4776,7 +4773,7 @@
         <v>435</v>
       </c>
       <c r="T53" s="2" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
     </row>
     <row r="54" spans="1:24" x14ac:dyDescent="0.3">
@@ -4817,7 +4814,7 @@
         <v>435</v>
       </c>
       <c r="T54" s="2" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
     </row>
     <row r="55" spans="1:24" x14ac:dyDescent="0.3">
@@ -4888,10 +4885,10 @@
         <v>435</v>
       </c>
       <c r="S56" s="2" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="T56" s="2" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
     </row>
     <row r="57" spans="1:24" x14ac:dyDescent="0.3">
@@ -4917,7 +4914,7 @@
         <v>1</v>
       </c>
       <c r="L57" s="3" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="M57" s="2" t="s">
         <v>352</v>
@@ -4947,7 +4944,7 @@
         <v>20</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="H58" s="2" t="s">
         <v>351</v>
@@ -4959,7 +4956,7 @@
         <v>2</v>
       </c>
       <c r="L58" s="2" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="M58" s="2" t="s">
         <v>351</v>
@@ -4971,10 +4968,10 @@
         <v>435</v>
       </c>
       <c r="T58" s="2" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="U58" s="2" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
     </row>
     <row r="59" spans="1:24" x14ac:dyDescent="0.3">
@@ -4994,7 +4991,7 @@
         <v>38</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="H59" s="2" t="s">
         <v>351</v>
@@ -5006,7 +5003,7 @@
         <v>3</v>
       </c>
       <c r="L59" s="2" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="M59" s="2" t="s">
         <v>351</v>
@@ -5018,7 +5015,7 @@
         <v>435</v>
       </c>
       <c r="T59" s="2" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
     </row>
     <row r="60" spans="1:24" x14ac:dyDescent="0.3">
@@ -5059,10 +5056,10 @@
         <v>435</v>
       </c>
       <c r="S60" s="2" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="T60" s="2" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
     </row>
     <row r="61" spans="1:24" x14ac:dyDescent="0.3">
@@ -5247,7 +5244,7 @@
         <v>2</v>
       </c>
       <c r="L65" s="2" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="M65" s="2" t="s">
         <v>351</v>
@@ -5259,7 +5256,7 @@
         <v>435</v>
       </c>
       <c r="T65" s="2" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="U65" s="2" t="s">
         <v>279</v>
@@ -5282,7 +5279,7 @@
         <v>24</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="H66" s="2" t="s">
         <v>351</v>
@@ -5294,7 +5291,7 @@
         <v>2</v>
       </c>
       <c r="L66" s="2" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="M66" s="2" t="s">
         <v>351</v>
@@ -5306,7 +5303,7 @@
         <v>435</v>
       </c>
       <c r="T66" s="2" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="U66" s="2" t="s">
         <v>276</v>
@@ -5329,7 +5326,7 @@
         <v>34</v>
       </c>
       <c r="G67" s="2" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="H67" s="2" t="s">
         <v>351</v>
@@ -5341,7 +5338,7 @@
         <v>3</v>
       </c>
       <c r="L67" s="3" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="M67" s="2" t="s">
         <v>351</v>
@@ -5353,10 +5350,10 @@
         <v>435</v>
       </c>
       <c r="T67" s="2" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="U67" s="2" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="68" spans="1:24" x14ac:dyDescent="0.3">
@@ -5376,7 +5373,7 @@
         <v>43</v>
       </c>
       <c r="G68" s="2" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="H68" s="2" t="s">
         <v>351</v>
@@ -5400,7 +5397,7 @@
         <v>435</v>
       </c>
       <c r="T68" s="2" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="U68" s="2" t="s">
         <v>232</v>
@@ -5423,7 +5420,7 @@
         <v>42</v>
       </c>
       <c r="G69" s="2" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="H69" s="2" t="s">
         <v>351</v>
@@ -5447,7 +5444,7 @@
         <v>435</v>
       </c>
       <c r="T69" s="2" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="U69" s="2" t="s">
         <v>280</v>
@@ -5470,7 +5467,7 @@
         <v>31</v>
       </c>
       <c r="G70" s="2" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="H70" s="2" t="s">
         <v>351</v>
@@ -5482,7 +5479,7 @@
         <v>3</v>
       </c>
       <c r="L70" s="3" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="M70" s="2" t="s">
         <v>351</v>
@@ -5494,7 +5491,7 @@
         <v>435</v>
       </c>
       <c r="T70" s="2" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="U70" s="2" t="s">
         <v>278</v>
@@ -5517,7 +5514,7 @@
         <v>45</v>
       </c>
       <c r="G71" s="2" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="H71" s="2" t="s">
         <v>351</v>
@@ -5529,7 +5526,7 @@
         <v>5</v>
       </c>
       <c r="L71" s="2" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="M71" s="2" t="s">
         <v>351</v>
@@ -5541,7 +5538,7 @@
         <v>435</v>
       </c>
       <c r="T71" s="2" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
     </row>
     <row r="72" spans="1:24" x14ac:dyDescent="0.3">
@@ -5561,10 +5558,10 @@
         <v>399</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="G72" s="2" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="H72" s="2" t="s">
         <v>351</v>
@@ -5585,10 +5582,10 @@
         <v>435</v>
       </c>
       <c r="T72" s="2" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="X72" s="2" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
     </row>
     <row r="73" spans="1:24" x14ac:dyDescent="0.3">
@@ -5608,10 +5605,10 @@
         <v>186</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="G73" s="2" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="H73" s="2" t="s">
         <v>351</v>
@@ -5623,7 +5620,7 @@
         <v>3</v>
       </c>
       <c r="L73" s="2" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="M73" s="2" t="s">
         <v>351</v>
@@ -5635,7 +5632,7 @@
         <v>435</v>
       </c>
       <c r="T73" s="2" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
     </row>
     <row r="74" spans="1:24" x14ac:dyDescent="0.3">
@@ -5676,10 +5673,10 @@
         <v>435</v>
       </c>
       <c r="S74" s="2" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="T74" s="2" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="75" spans="1:24" x14ac:dyDescent="0.3">
@@ -5714,10 +5711,10 @@
         <v>435</v>
       </c>
       <c r="S75" s="2" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="T75" s="2" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
     </row>
     <row r="76" spans="1:24" x14ac:dyDescent="0.3">
@@ -5755,7 +5752,7 @@
         <v>435</v>
       </c>
       <c r="T76" s="2" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="X76" s="2" t="s">
         <v>184</v>
@@ -5778,10 +5775,10 @@
         <v>48</v>
       </c>
       <c r="F77" s="2" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="G77" s="2" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="H77" s="2" t="s">
         <v>351</v>
@@ -5793,7 +5790,7 @@
         <v>4</v>
       </c>
       <c r="L77" s="3" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="M77" s="2" t="s">
         <v>351</v>
@@ -5805,7 +5802,7 @@
         <v>435</v>
       </c>
       <c r="T77" s="2" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
     </row>
     <row r="78" spans="1:24" x14ac:dyDescent="0.3">
@@ -5825,10 +5822,10 @@
         <v>47</v>
       </c>
       <c r="F78" s="2" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="G78" s="2" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="H78" s="2" t="s">
         <v>351</v>
@@ -5840,7 +5837,7 @@
         <v>5</v>
       </c>
       <c r="L78" s="3" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="M78" s="2" t="s">
         <v>351</v>
@@ -5852,7 +5849,7 @@
         <v>435</v>
       </c>
       <c r="T78" s="2" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
     </row>
     <row r="79" spans="1:24" x14ac:dyDescent="0.3">
@@ -5869,7 +5866,7 @@
         <v>138</v>
       </c>
       <c r="F79" s="2" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="H79" s="2" t="s">
         <v>351</v>
@@ -5881,7 +5878,7 @@
         <v>6</v>
       </c>
       <c r="L79" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="M79" s="2" t="s">
         <v>351</v>
@@ -5893,10 +5890,10 @@
         <v>435</v>
       </c>
       <c r="S79" s="2" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="T79" s="2" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
     </row>
     <row r="80" spans="1:24" x14ac:dyDescent="0.3">
@@ -5934,7 +5931,7 @@
         <v>435</v>
       </c>
       <c r="T80" s="2" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="X80" s="2" t="s">
         <v>163</v>
@@ -5963,7 +5960,7 @@
         <v>4</v>
       </c>
       <c r="L81" s="3" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="M81" s="3" t="s">
         <v>351</v>
@@ -5975,7 +5972,7 @@
         <v>435</v>
       </c>
       <c r="T81" s="2" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
     </row>
     <row r="82" spans="1:24" ht="43.2" x14ac:dyDescent="0.3">
@@ -6004,7 +6001,7 @@
         <v>4</v>
       </c>
       <c r="L82" s="3" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="M82" s="2" t="s">
         <v>351</v>
@@ -6016,7 +6013,7 @@
         <v>435</v>
       </c>
       <c r="T82" s="2" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
     </row>
     <row r="83" spans="1:24" ht="115.2" x14ac:dyDescent="0.3">
@@ -6084,10 +6081,10 @@
         <v>435</v>
       </c>
       <c r="S84" s="2" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="T84" s="2" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="85" spans="1:24" x14ac:dyDescent="0.3">
@@ -6215,7 +6212,7 @@
         <v>1</v>
       </c>
       <c r="L88" s="3" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="M88" s="2" t="s">
         <v>351</v>
@@ -6226,8 +6223,8 @@
       <c r="O88" s="2" t="s">
         <v>435</v>
       </c>
-      <c r="T88" s="15" t="s">
-        <v>674</v>
+      <c r="T88" s="12" t="s">
+        <v>673</v>
       </c>
     </row>
     <row r="89" spans="1:24" x14ac:dyDescent="0.3">
@@ -6264,8 +6261,8 @@
       <c r="O89" s="2" t="s">
         <v>435</v>
       </c>
-      <c r="T89" s="15" t="s">
-        <v>675</v>
+      <c r="T89" s="12" t="s">
+        <v>674</v>
       </c>
     </row>
     <row r="90" spans="1:24" x14ac:dyDescent="0.3">
@@ -6302,8 +6299,8 @@
       <c r="O90" s="2" t="s">
         <v>435</v>
       </c>
-      <c r="T90" s="15" t="s">
-        <v>675</v>
+      <c r="T90" s="12" t="s">
+        <v>674</v>
       </c>
     </row>
     <row r="91" spans="1:24" x14ac:dyDescent="0.3">
@@ -6343,8 +6340,8 @@
       <c r="O91" s="2" t="s">
         <v>435</v>
       </c>
-      <c r="T91" s="15" t="s">
-        <v>676</v>
+      <c r="T91" s="12" t="s">
+        <v>675</v>
       </c>
     </row>
     <row r="92" spans="1:24" x14ac:dyDescent="0.3">
@@ -6361,7 +6358,7 @@
         <v>351</v>
       </c>
       <c r="L92" s="2" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="M92" s="2" t="s">
         <v>352</v>
@@ -6403,7 +6400,7 @@
         <v>6</v>
       </c>
       <c r="L93" s="2" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="M93" s="2" t="s">
         <v>351</v>
@@ -6415,7 +6412,7 @@
         <v>435</v>
       </c>
       <c r="T93" s="2" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
     </row>
     <row r="94" spans="1:24" x14ac:dyDescent="0.3">
@@ -6435,10 +6432,10 @@
         <v>23</v>
       </c>
       <c r="F94" s="2" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="G94" s="2" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="H94" s="2" t="s">
         <v>351</v>
@@ -6450,7 +6447,7 @@
         <v>2</v>
       </c>
       <c r="L94" s="2" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="M94" s="2" t="s">
         <v>351</v>
@@ -6462,10 +6459,10 @@
         <v>435</v>
       </c>
       <c r="T94" s="2" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="U94" s="2" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="X94" s="2" t="s">
         <v>158</v>
@@ -6488,7 +6485,7 @@
         <v>44</v>
       </c>
       <c r="G95" s="2" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="H95" s="2" t="s">
         <v>351</v>
@@ -6500,7 +6497,7 @@
         <v>5</v>
       </c>
       <c r="L95" s="2" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="M95" s="2" t="s">
         <v>351</v>
@@ -6512,7 +6509,7 @@
         <v>435</v>
       </c>
       <c r="T95" s="2" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
     </row>
     <row r="96" spans="1:24" x14ac:dyDescent="0.3">
@@ -6571,7 +6568,7 @@
         <v>444</v>
       </c>
       <c r="L97" s="3" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="M97" s="3" t="s">
         <v>351</v>
@@ -6583,7 +6580,7 @@
         <v>435</v>
       </c>
       <c r="T97" s="2" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
     </row>
     <row r="98" spans="1:24" x14ac:dyDescent="0.3">
@@ -6618,10 +6615,10 @@
         <v>435</v>
       </c>
       <c r="S98" s="2" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="T98" s="2" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="99" spans="1:24" x14ac:dyDescent="0.3">
@@ -6650,7 +6647,7 @@
         <v>2</v>
       </c>
       <c r="L99" s="2" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="M99" s="2" t="s">
         <v>351</v>
@@ -6665,7 +6662,7 @@
         <v>447</v>
       </c>
       <c r="T99" s="2" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
     </row>
     <row r="100" spans="1:24" x14ac:dyDescent="0.3">
@@ -6706,7 +6703,7 @@
         <v>435</v>
       </c>
       <c r="T100" s="2" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
     </row>
     <row r="101" spans="1:24" x14ac:dyDescent="0.3">
@@ -6732,7 +6729,7 @@
         <v>5</v>
       </c>
       <c r="L101" s="3" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="M101" s="2" t="s">
         <v>351</v>
@@ -6744,7 +6741,7 @@
         <v>435</v>
       </c>
       <c r="T101" s="2" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
     </row>
     <row r="102" spans="1:24" x14ac:dyDescent="0.3">
@@ -6770,7 +6767,7 @@
         <v>4</v>
       </c>
       <c r="L102" s="2" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="M102" s="2" t="s">
         <v>351</v>
@@ -6782,7 +6779,7 @@
         <v>435</v>
       </c>
       <c r="T102" s="2" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
     </row>
     <row r="103" spans="1:24" x14ac:dyDescent="0.3">
@@ -6823,7 +6820,7 @@
         <v>435</v>
       </c>
       <c r="T103" s="2" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
     </row>
     <row r="104" spans="1:24" x14ac:dyDescent="0.3">
@@ -6864,10 +6861,10 @@
         <v>447</v>
       </c>
       <c r="S104" s="2" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="T104" s="2" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="X104" s="2" t="s">
         <v>166</v>
@@ -6886,10 +6883,10 @@
       <c r="H105" s="2" t="s">
         <v>351</v>
       </c>
-      <c r="L105" s="11" t="s">
+      <c r="L105" s="8" t="s">
         <v>354</v>
       </c>
-      <c r="M105" s="13" t="s">
+      <c r="M105" s="10" t="s">
         <v>352</v>
       </c>
       <c r="N105" s="2" t="s">
@@ -6932,7 +6929,7 @@
         <v>4</v>
       </c>
       <c r="L106" s="3" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="M106" s="2" t="s">
         <v>351</v>
@@ -6944,7 +6941,7 @@
         <v>435</v>
       </c>
       <c r="T106" s="2" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="X106" s="2" t="s">
         <v>161</v>
@@ -6976,7 +6973,7 @@
         <v>5</v>
       </c>
       <c r="L107" s="3" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="M107" s="2" t="s">
         <v>351</v>
@@ -6988,7 +6985,7 @@
         <v>435</v>
       </c>
       <c r="T107" s="2" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="X107" s="2" t="s">
         <v>430</v>
@@ -7020,7 +7017,7 @@
         <v>6</v>
       </c>
       <c r="L108" s="2" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="M108" s="2" t="s">
         <v>351</v>
@@ -7035,7 +7032,7 @@
         <v>447</v>
       </c>
       <c r="T108" s="2" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="X108" s="2" t="s">
         <v>161</v>
@@ -7064,7 +7061,7 @@
         <v>6</v>
       </c>
       <c r="L109" s="3" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="M109" s="2" t="s">
         <v>351</v>
@@ -7076,7 +7073,7 @@
         <v>435</v>
       </c>
       <c r="T109" s="2" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
     </row>
     <row r="110" spans="1:24" x14ac:dyDescent="0.3">
@@ -7101,10 +7098,10 @@
       <c r="K110" s="2">
         <v>7</v>
       </c>
-      <c r="L110" s="9" t="s">
-        <v>589</v>
-      </c>
-      <c r="M110" s="10" t="s">
+      <c r="L110" s="7" t="s">
+        <v>588</v>
+      </c>
+      <c r="M110" s="2" t="s">
         <v>351</v>
       </c>
       <c r="N110" s="2" t="s">
@@ -7114,10 +7111,10 @@
         <v>435</v>
       </c>
       <c r="S110" s="2" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="T110" s="2" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="111" spans="1:24" x14ac:dyDescent="0.3">
@@ -7143,7 +7140,7 @@
         <v>4</v>
       </c>
       <c r="L111" s="2" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="M111" s="2" t="s">
         <v>351</v>
@@ -7155,7 +7152,7 @@
         <v>435</v>
       </c>
       <c r="T111" s="2" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
     </row>
     <row r="112" spans="1:24" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7182,7 +7179,7 @@
         <v>3</v>
       </c>
       <c r="L112" s="2" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="M112" s="2" t="s">
         <v>351</v>
@@ -7194,7 +7191,7 @@
         <v>435</v>
       </c>
       <c r="T112" s="2" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="U112" s="2" t="s">
         <v>319</v>
@@ -7250,7 +7247,7 @@
         <v>191</v>
       </c>
       <c r="E114" s="2" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="H114" s="2" t="s">
         <v>351</v>
@@ -7262,7 +7259,7 @@
         <v>1</v>
       </c>
       <c r="L114" s="3" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="M114" s="2" t="s">
         <v>352</v>
@@ -7298,7 +7295,7 @@
         <v>1</v>
       </c>
       <c r="L115" s="3" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="M115" s="3" t="s">
         <v>351</v>
@@ -7309,8 +7306,8 @@
       <c r="O115" s="2" t="s">
         <v>435</v>
       </c>
-      <c r="T115" s="15" t="s">
-        <v>673</v>
+      <c r="T115" s="12" t="s">
+        <v>672</v>
       </c>
       <c r="X115" s="2" t="s">
         <v>474</v>
@@ -7333,7 +7330,7 @@
         <v>78</v>
       </c>
       <c r="G116" s="2" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="H116" s="2" t="s">
         <v>351</v>
@@ -7357,7 +7354,7 @@
         <v>435</v>
       </c>
       <c r="T116" s="2" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
     </row>
     <row r="117" spans="1:24" x14ac:dyDescent="0.3">
@@ -7450,7 +7447,7 @@
         <v>435</v>
       </c>
       <c r="T119" s="2" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="X119" s="2" t="s">
         <v>183</v>
@@ -7473,7 +7470,7 @@
         <v>39</v>
       </c>
       <c r="G120" s="2" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="H120" s="2" t="s">
         <v>351</v>
@@ -7485,7 +7482,7 @@
         <v>3</v>
       </c>
       <c r="L120" s="3" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="M120" s="2" t="s">
         <v>351</v>
@@ -7497,7 +7494,7 @@
         <v>435</v>
       </c>
       <c r="T120" s="2" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
     </row>
     <row r="121" spans="1:24" x14ac:dyDescent="0.3">
@@ -7523,7 +7520,7 @@
         <v>4</v>
       </c>
       <c r="L121" s="2" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="M121" s="2" t="s">
         <v>351</v>
@@ -7535,7 +7532,7 @@
         <v>435</v>
       </c>
       <c r="T121" s="2" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
     </row>
     <row r="122" spans="1:24" x14ac:dyDescent="0.3">
@@ -7596,10 +7593,10 @@
       <c r="K123" s="2">
         <v>5</v>
       </c>
-      <c r="L123" s="8" t="s">
+      <c r="L123" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="M123" s="8" t="s">
+      <c r="M123" s="4" t="s">
         <v>351</v>
       </c>
       <c r="N123" s="2" t="s">
@@ -7609,7 +7606,7 @@
         <v>435</v>
       </c>
       <c r="T123" s="2" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
     </row>
     <row r="124" spans="1:24" x14ac:dyDescent="0.3">
@@ -7629,10 +7626,10 @@
         <v>70</v>
       </c>
       <c r="F124" s="2" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="G124" s="2" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="H124" s="2" t="s">
         <v>351</v>
@@ -7644,7 +7641,7 @@
         <v>4</v>
       </c>
       <c r="L124" s="3" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="M124" s="2" t="s">
         <v>351</v>
@@ -7656,7 +7653,7 @@
         <v>435</v>
       </c>
       <c r="T124" s="2" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
     </row>
     <row r="125" spans="1:24" x14ac:dyDescent="0.3">
@@ -7676,7 +7673,7 @@
         <v>72</v>
       </c>
       <c r="G125" s="2" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="H125" s="2" t="s">
         <v>351</v>
@@ -7688,7 +7685,7 @@
         <v>5</v>
       </c>
       <c r="L125" s="2" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="M125" s="2" t="s">
         <v>351</v>
@@ -7700,7 +7697,7 @@
         <v>435</v>
       </c>
       <c r="T125" s="2" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="X125" s="2" t="s">
         <v>372</v>
@@ -7723,7 +7720,7 @@
         <v>74</v>
       </c>
       <c r="G126" s="2" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="H126" s="2" t="s">
         <v>351</v>
@@ -7735,7 +7732,7 @@
         <v>6</v>
       </c>
       <c r="L126" s="2" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="M126" s="2" t="s">
         <v>351</v>
@@ -7747,7 +7744,7 @@
         <v>435</v>
       </c>
       <c r="T126" s="2" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
     </row>
     <row r="127" spans="1:24" ht="86.4" x14ac:dyDescent="0.3">
@@ -7809,7 +7806,7 @@
         <v>6</v>
       </c>
       <c r="L128" s="2" t="s">
-        <v>494</v>
+        <v>698</v>
       </c>
       <c r="M128" s="2" t="s">
         <v>351</v>
@@ -7821,7 +7818,7 @@
         <v>435</v>
       </c>
       <c r="T128" s="2" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
     </row>
     <row r="129" spans="1:24" x14ac:dyDescent="0.3">
@@ -7856,7 +7853,7 @@
         <v>435</v>
       </c>
       <c r="T129" s="2" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
     </row>
     <row r="130" spans="1:24" x14ac:dyDescent="0.3">
@@ -7876,7 +7873,7 @@
         <v>79</v>
       </c>
       <c r="G130" s="2" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="H130" s="2" t="s">
         <v>351</v>
@@ -7888,7 +7885,7 @@
         <v>4</v>
       </c>
       <c r="L130" s="2" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="M130" s="2" t="s">
         <v>351</v>
@@ -7900,7 +7897,7 @@
         <v>435</v>
       </c>
       <c r="T130" s="2" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
     </row>
     <row r="131" spans="1:24" x14ac:dyDescent="0.3">
@@ -7920,7 +7917,7 @@
         <v>80</v>
       </c>
       <c r="G131" s="2" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="H131" s="2" t="s">
         <v>351</v>
@@ -7932,7 +7929,7 @@
         <v>5</v>
       </c>
       <c r="L131" s="2" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="M131" s="2" t="s">
         <v>351</v>
@@ -7944,7 +7941,7 @@
         <v>435</v>
       </c>
       <c r="T131" s="2" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
     </row>
     <row r="132" spans="1:24" x14ac:dyDescent="0.3">
@@ -7967,7 +7964,7 @@
         <v>433</v>
       </c>
       <c r="G132" s="2" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="H132" s="2" t="s">
         <v>351</v>
@@ -7979,7 +7976,7 @@
         <v>6</v>
       </c>
       <c r="L132" s="2" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="M132" s="2" t="s">
         <v>351</v>
@@ -7994,7 +7991,7 @@
         <v>447</v>
       </c>
       <c r="T132" s="2" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
     </row>
     <row r="133" spans="1:24" x14ac:dyDescent="0.3">
@@ -8010,10 +8007,9 @@
       <c r="E133" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="F133" s="10" t="s">
+      <c r="F133" s="2" t="s">
         <v>408</v>
       </c>
-      <c r="G133" s="10"/>
       <c r="H133" s="2" t="s">
         <v>351</v>
       </c>
@@ -8036,7 +8032,7 @@
         <v>435</v>
       </c>
       <c r="T133" s="2" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
     </row>
     <row r="134" spans="1:24" x14ac:dyDescent="0.3">
@@ -8055,8 +8051,7 @@
       <c r="E134" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="F134" s="10"/>
-      <c r="G134" s="10" t="s">
+      <c r="G134" s="2" t="s">
         <v>492</v>
       </c>
       <c r="H134" s="2" t="s">
@@ -8078,7 +8073,7 @@
         <v>435</v>
       </c>
       <c r="T134" s="2" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
     </row>
     <row r="135" spans="1:24" x14ac:dyDescent="0.3">
@@ -8094,14 +8089,14 @@
       <c r="D135" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="E135" s="7" t="s">
+      <c r="E135" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="F135" s="10" t="s">
+      <c r="F135" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="G135" s="10" t="s">
-        <v>544</v>
+      <c r="G135" s="2" t="s">
+        <v>543</v>
       </c>
       <c r="H135" s="2" t="s">
         <v>351</v>
@@ -8113,7 +8108,7 @@
         <v>3</v>
       </c>
       <c r="L135" s="3" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="M135" s="2" t="s">
         <v>351</v>
@@ -8125,10 +8120,10 @@
         <v>435</v>
       </c>
       <c r="T135" s="2" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="U135" s="2" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
     </row>
     <row r="136" spans="1:24" x14ac:dyDescent="0.3">
@@ -8205,7 +8200,7 @@
         <v>435</v>
       </c>
       <c r="T137" s="2" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
     </row>
     <row r="138" spans="1:24" x14ac:dyDescent="0.3">
@@ -8276,10 +8271,10 @@
         <v>435</v>
       </c>
       <c r="S139" s="2" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="T139" s="2" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="140" spans="1:24" x14ac:dyDescent="0.3">
@@ -8296,7 +8291,7 @@
         <v>5</v>
       </c>
       <c r="F140" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="H140" s="2" t="s">
         <v>351</v>
@@ -8308,7 +8303,7 @@
         <v>1</v>
       </c>
       <c r="L140" s="3" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="M140" s="2" t="s">
         <v>351</v>
@@ -8319,8 +8314,8 @@
       <c r="O140" s="2" t="s">
         <v>435</v>
       </c>
-      <c r="T140" s="15" t="s">
-        <v>647</v>
+      <c r="T140" s="12" t="s">
+        <v>646</v>
       </c>
     </row>
     <row r="141" spans="1:24" x14ac:dyDescent="0.3">
@@ -8346,7 +8341,7 @@
         <v>4</v>
       </c>
       <c r="L141" s="3" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="M141" s="3" t="s">
         <v>351</v>
@@ -8358,7 +8353,7 @@
         <v>435</v>
       </c>
       <c r="T141" s="2" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="X141" s="2" t="s">
         <v>194</v>
@@ -8396,7 +8391,7 @@
         <v>435</v>
       </c>
       <c r="T142" s="2"/>
-      <c r="X142" s="12" t="s">
+      <c r="X142" s="9" t="s">
         <v>360</v>
       </c>
     </row>
@@ -8584,7 +8579,7 @@
         <v>403</v>
       </c>
       <c r="F148" s="2" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="H148" s="2" t="s">
         <v>351</v>
@@ -8596,7 +8591,7 @@
         <v>405</v>
       </c>
       <c r="L148" s="2" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="M148" s="2" t="s">
         <v>351</v>
@@ -8608,7 +8603,7 @@
         <v>435</v>
       </c>
       <c r="T148" s="2" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
     </row>
     <row r="149" spans="1:24" x14ac:dyDescent="0.3">
@@ -8775,7 +8770,7 @@
         <v>436</v>
       </c>
       <c r="S153" s="2" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="T153" s="2"/>
     </row>
@@ -8832,13 +8827,13 @@
         <v>352</v>
       </c>
       <c r="O155" s="2" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="T155" s="2"/>
     </row>
     <row r="156" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A156" s="2" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="B156" s="2" t="s">
         <v>124</v>
@@ -8850,42 +8845,42 @@
         <v>138</v>
       </c>
       <c r="F156" s="2" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="H156" s="2" t="s">
         <v>351</v>
       </c>
       <c r="I156" s="2" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="K156" s="2">
         <v>6</v>
       </c>
       <c r="L156" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="M156" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="N156" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="O156" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="S156" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="T156" s="2" t="s">
+        <v>667</v>
+      </c>
+      <c r="X156" s="2" t="s">
         <v>580</v>
-      </c>
-      <c r="M156" s="2" t="s">
-        <v>351</v>
-      </c>
-      <c r="N156" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="O156" s="2" t="s">
-        <v>435</v>
-      </c>
-      <c r="S156" s="2" t="s">
-        <v>597</v>
-      </c>
-      <c r="T156" s="2" t="s">
-        <v>668</v>
-      </c>
-      <c r="X156" s="2" t="s">
-        <v>581</v>
       </c>
     </row>
     <row r="157" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A157" s="2" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="B157" s="2" t="s">
         <v>18</v>
@@ -8894,10 +8889,10 @@
         <v>191</v>
       </c>
       <c r="E157" s="2" t="s">
+        <v>610</v>
+      </c>
+      <c r="F157" s="2" t="s">
         <v>611</v>
-      </c>
-      <c r="F157" s="2" t="s">
-        <v>612</v>
       </c>
       <c r="H157" s="2" t="s">
         <v>351</v>
@@ -8909,7 +8904,7 @@
         <v>361</v>
       </c>
       <c r="L157" s="2" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="M157" s="2" t="s">
         <v>352</v>
@@ -8922,30 +8917,30 @@
       </c>
       <c r="T157" s="2"/>
       <c r="X157" s="2" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
     </row>
     <row r="158" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A158" s="2" t="s">
+        <v>614</v>
+      </c>
+      <c r="B158" s="2" t="s">
         <v>615</v>
       </c>
-      <c r="B158" s="2" t="s">
+      <c r="D158" s="2" t="s">
         <v>616</v>
       </c>
-      <c r="D158" s="2" t="s">
+      <c r="E158" s="2" t="s">
         <v>617</v>
       </c>
-      <c r="E158" s="2" t="s">
+      <c r="H158" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="L158" s="2" t="s">
+        <v>680</v>
+      </c>
+      <c r="M158" s="2" t="s">
         <v>618</v>
-      </c>
-      <c r="H158" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="L158" s="2" t="s">
-        <v>681</v>
-      </c>
-      <c r="M158" s="2" t="s">
-        <v>619</v>
       </c>
       <c r="N158" s="2" t="s">
         <v>352</v>
@@ -8955,21 +8950,21 @@
       </c>
       <c r="T158" s="2"/>
       <c r="V158" s="2" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="X158" s="2" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
     </row>
     <row r="159" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A159" s="2" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="B159" s="2" t="s">
         <v>477</v>
       </c>
       <c r="E159" s="2" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="H159" s="2" t="s">
         <v>352</v>
@@ -8978,40 +8973,40 @@
         <v>396</v>
       </c>
       <c r="L159" s="2" t="s">
+        <v>622</v>
+      </c>
+      <c r="M159" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="N159" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="O159" s="2" t="s">
         <v>623</v>
-      </c>
-      <c r="M159" s="2" t="s">
-        <v>351</v>
-      </c>
-      <c r="N159" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="O159" s="2" t="s">
-        <v>624</v>
       </c>
       <c r="T159" s="2"/>
     </row>
     <row r="160" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A160" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="B160" s="2" t="s">
+        <v>615</v>
+      </c>
+      <c r="D160" s="2" t="s">
+        <v>616</v>
+      </c>
+      <c r="E160" s="2" t="s">
         <v>682</v>
       </c>
-      <c r="B160" s="2" t="s">
-        <v>616</v>
-      </c>
-      <c r="D160" s="2" t="s">
-        <v>617</v>
-      </c>
-      <c r="E160" s="2" t="s">
-        <v>683</v>
-      </c>
       <c r="H160" s="2" t="s">
         <v>352</v>
       </c>
       <c r="L160" s="2" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="M160" s="2" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="N160" s="2" t="s">
         <v>352</v>
@@ -9020,30 +9015,30 @@
         <v>435</v>
       </c>
       <c r="V160" s="2" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
     </row>
     <row r="161" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A161" s="2" t="s">
+        <v>683</v>
+      </c>
+      <c r="B161" s="2" t="s">
+        <v>615</v>
+      </c>
+      <c r="D161" s="2" t="s">
+        <v>616</v>
+      </c>
+      <c r="E161" s="2" t="s">
         <v>684</v>
       </c>
-      <c r="B161" s="2" t="s">
-        <v>616</v>
-      </c>
-      <c r="D161" s="2" t="s">
-        <v>617</v>
-      </c>
-      <c r="E161" s="2" t="s">
+      <c r="H161" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="L161" s="2" t="s">
         <v>685</v>
       </c>
-      <c r="H161" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="L161" s="2" t="s">
-        <v>686</v>
-      </c>
       <c r="M161" s="2" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="N161" s="2" t="s">
         <v>352</v>
@@ -9052,30 +9047,30 @@
         <v>435</v>
       </c>
       <c r="V161" s="2" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
     </row>
     <row r="162" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A162" s="2" t="s">
+        <v>686</v>
+      </c>
+      <c r="B162" s="2" t="s">
+        <v>615</v>
+      </c>
+      <c r="D162" s="2" t="s">
+        <v>616</v>
+      </c>
+      <c r="E162" s="2" t="s">
         <v>687</v>
       </c>
-      <c r="B162" s="2" t="s">
-        <v>616</v>
-      </c>
-      <c r="D162" s="2" t="s">
-        <v>617</v>
-      </c>
-      <c r="E162" s="2" t="s">
-        <v>688</v>
-      </c>
       <c r="H162" s="2" t="s">
         <v>352</v>
       </c>
       <c r="L162" s="2" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="M162" s="2" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="N162" s="2" t="s">
         <v>352</v>
@@ -9084,30 +9079,30 @@
         <v>435</v>
       </c>
       <c r="V162" s="2" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
     </row>
     <row r="163" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A163" s="2" t="s">
+        <v>688</v>
+      </c>
+      <c r="B163" s="2" t="s">
+        <v>615</v>
+      </c>
+      <c r="D163" s="2" t="s">
+        <v>616</v>
+      </c>
+      <c r="E163" s="2" t="s">
         <v>689</v>
       </c>
-      <c r="B163" s="2" t="s">
-        <v>616</v>
-      </c>
-      <c r="D163" s="2" t="s">
-        <v>617</v>
-      </c>
-      <c r="E163" s="2" t="s">
-        <v>690</v>
-      </c>
       <c r="H163" s="2" t="s">
         <v>352</v>
       </c>
       <c r="L163" s="2" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="M163" s="2" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="N163" s="2" t="s">
         <v>352</v>
@@ -9116,30 +9111,30 @@
         <v>435</v>
       </c>
       <c r="V163" s="2" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
     </row>
     <row r="164" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A164" s="2" t="s">
+        <v>690</v>
+      </c>
+      <c r="B164" s="2" t="s">
+        <v>615</v>
+      </c>
+      <c r="D164" s="2" t="s">
+        <v>616</v>
+      </c>
+      <c r="E164" s="2" t="s">
         <v>691</v>
       </c>
-      <c r="B164" s="2" t="s">
-        <v>616</v>
-      </c>
-      <c r="D164" s="2" t="s">
-        <v>617</v>
-      </c>
-      <c r="E164" s="2" t="s">
-        <v>692</v>
-      </c>
       <c r="H164" s="2" t="s">
         <v>352</v>
       </c>
       <c r="L164" s="2" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="M164" s="2" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="N164" s="2" t="s">
         <v>352</v>
@@ -9148,30 +9143,30 @@
         <v>435</v>
       </c>
       <c r="V164" s="2" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
     <row r="165" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A165" s="2" t="s">
+        <v>693</v>
+      </c>
+      <c r="B165" s="2" t="s">
+        <v>615</v>
+      </c>
+      <c r="D165" s="2" t="s">
+        <v>616</v>
+      </c>
+      <c r="E165" s="2" t="s">
         <v>694</v>
       </c>
-      <c r="B165" s="2" t="s">
-        <v>616</v>
-      </c>
-      <c r="D165" s="2" t="s">
-        <v>617</v>
-      </c>
-      <c r="E165" s="2" t="s">
-        <v>695</v>
-      </c>
       <c r="H165" s="2" t="s">
         <v>352</v>
       </c>
       <c r="L165" s="2" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="M165" s="2" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="N165" s="2" t="s">
         <v>352</v>
@@ -9180,30 +9175,30 @@
         <v>435</v>
       </c>
       <c r="V165" s="2" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
     <row r="166" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A166" s="2" t="s">
+        <v>695</v>
+      </c>
+      <c r="B166" s="2" t="s">
+        <v>615</v>
+      </c>
+      <c r="D166" s="2" t="s">
+        <v>616</v>
+      </c>
+      <c r="E166" s="2" t="s">
         <v>696</v>
       </c>
-      <c r="B166" s="2" t="s">
-        <v>616</v>
-      </c>
-      <c r="D166" s="2" t="s">
-        <v>617</v>
-      </c>
-      <c r="E166" s="2" t="s">
-        <v>697</v>
-      </c>
       <c r="H166" s="2" t="s">
         <v>352</v>
       </c>
       <c r="L166" s="2" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="M166" s="2" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="N166" s="2" t="s">
         <v>352</v>
@@ -9212,11 +9207,11 @@
         <v>435</v>
       </c>
       <c r="V166" s="2" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Y159" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:Y166" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:O146">
     <sortCondition ref="E2:E146"/>
     <sortCondition ref="I2:I146"/>

</xml_diff>